<commit_message>
deploy: feature/careteam → branches/feature-careteam 0f7b126ed7a7abe52cc3965a42f4ee56eae05f45
</commit_message>
<xml_diff>
--- a/branches/feature-careteam/StructureDefinition-RIVManagingTeam-careteam.xlsx
+++ b/branches/feature-careteam/StructureDefinition-RIVManagingTeam-careteam.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-11T07:06:47+00:00</t>
+    <t>2026-09-21T07:30:27+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -885,7 +885,7 @@
 ctm-2</t>
   </si>
   <si>
-    <t>Personal.id,Personal.namn,Personal.befattning</t>
+    <t>Personal</t>
   </si>
   <si>
     <t>FiveWs.actor</t>

</xml_diff>